<commit_message>
trips: payout disbursement panels + Step-16 payout Notes
- Rework Proxy and Carrier "Your Disbursement" panels to the requested layout:
  itemised due (Products+Margin / Carry Fee, Platform Fee in parens, Customs
  Duty Reimbursement), Total Due to You, then a "Payout Disbursed (…) Released
  on {date}" line and "Outstanding -" once paid, plus a centered "View Transfer
  Proof" button. Carrier now sees their payout proof (parity with Proxy).
- Add Step-16 (admin "Process Payout Disbursements") to the CLEAR Notes: once
  paid, Carrier/Proxy show "Your payout has been processed on {date}. Thank you
  for doing business with ProxyBuying." and the Buyer shows the disbursed-record
  note; gated on traveler_paid_at / proxy_disbursed_at so Notes update at payout
  rather than waiting for the close_cleared cron.
- Grammar fix on the Step-15.1 buyer clear line.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proxybuying-obsidian/AI-Context/references/UserAndSystemStepsRelationship.xlsx
+++ b/proxybuying-obsidian/AI-Context/references/UserAndSystemStepsRelationship.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="114">
   <si>
     <t xml:space="preserve">USERS AND SYSTEM STEPS RELATIONSHIP</t>
   </si>
@@ -326,6 +326,15 @@
   </si>
   <si>
     <t xml:space="preserve">Package received confirmed by the Buyer. Your payout will be disbursed within 24 hours.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Process Payout Disbursements</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For your record, Carrier and Proxy Buyer payouts have been disbursed on &lt;date, time&gt; </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Your payout has been processed on &lt;date, time&gt;. Thank you for doing business with ProxyBuying</t>
   </si>
   <si>
     <t xml:space="preserve">BUYER SELECTED: PICKUP THE PACKAGE</t>
@@ -442,7 +451,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -526,6 +535,9 @@
     </xf>
     <xf fontId="1" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="164" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1693,89 +1705,112 @@
         <v>102</v>
       </c>
     </row>
-    <row r="34" ht="14.25">
-      <c r="A34" s="9"/>
-      <c r="B34" s="9"/>
-      <c r="C34" s="9"/>
-      <c r="D34" s="10"/>
-      <c r="E34" s="23"/>
-      <c r="F34" s="23"/>
-      <c r="G34" s="23"/>
+    <row r="34" ht="57">
+      <c r="A34" s="9">
+        <v>16</v>
+      </c>
+      <c r="B34" s="18">
+        <v>16</v>
+      </c>
+      <c r="C34" s="30" t="s">
+        <v>47</v>
+      </c>
+      <c r="D34" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="E34" s="22" t="s">
+        <v>104</v>
+      </c>
+      <c r="F34" s="22" t="s">
+        <v>105</v>
+      </c>
+      <c r="G34" s="22" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="35" ht="14.25">
-      <c r="A35" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="B35" s="6"/>
-      <c r="C35" s="6"/>
-      <c r="D35" s="6"/>
-      <c r="E35" s="6"/>
-      <c r="F35" s="6"/>
-      <c r="G35" s="6"/>
+      <c r="A35" s="9"/>
+      <c r="B35" s="9"/>
+      <c r="C35" s="9"/>
+      <c r="D35" s="10"/>
+      <c r="E35" s="23"/>
+      <c r="F35" s="23"/>
+      <c r="G35" s="23"/>
     </row>
     <row r="36" ht="14.25">
-      <c r="A36" s="26"/>
-      <c r="B36" s="23"/>
-      <c r="C36" s="23"/>
-      <c r="D36" s="27"/>
-      <c r="E36" s="23"/>
-      <c r="F36" s="23"/>
-      <c r="G36" s="23"/>
-    </row>
-    <row r="37" ht="57">
-      <c r="A37" s="30" t="s">
-        <v>104</v>
-      </c>
-      <c r="B37" s="30" t="s">
-        <v>104</v>
-      </c>
-      <c r="C37" s="9" t="s">
+      <c r="A36" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B36" s="6"/>
+      <c r="C36" s="6"/>
+      <c r="D36" s="6"/>
+      <c r="E36" s="6"/>
+      <c r="F36" s="6"/>
+      <c r="G36" s="6"/>
+    </row>
+    <row r="37" ht="14.25">
+      <c r="A37" s="26"/>
+      <c r="B37" s="23"/>
+      <c r="C37" s="23"/>
+      <c r="D37" s="27"/>
+      <c r="E37" s="23"/>
+      <c r="F37" s="23"/>
+      <c r="G37" s="23"/>
+    </row>
+    <row r="38" ht="57">
+      <c r="A38" s="31" t="s">
+        <v>107</v>
+      </c>
+      <c r="B38" s="31" t="s">
+        <v>107</v>
+      </c>
+      <c r="C38" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D37" s="10" t="s">
+      <c r="D38" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="E37" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="F37" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="G37" s="12" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="38" ht="42.75">
-      <c r="A38" s="26" t="s">
+      <c r="E38" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="B38" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="C38" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="D38" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="E38" s="12" t="s">
+      <c r="F38" s="12" t="s">
         <v>109</v>
-      </c>
-      <c r="F38" s="12" t="s">
-        <v>110</v>
       </c>
       <c r="G38" s="12" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="39" ht="14.25">
-      <c r="A39" s="31"/>
-      <c r="B39" s="32"/>
-      <c r="C39" s="32"/>
-      <c r="D39" s="33"/>
-      <c r="E39" s="32"/>
-      <c r="F39" s="32"/>
-      <c r="G39" s="32"/>
+    <row r="39" ht="42.75">
+      <c r="A39" s="26" t="s">
+        <v>111</v>
+      </c>
+      <c r="B39" s="26" t="s">
+        <v>111</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="D39" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="E39" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="F39" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="G39" s="12" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="40" ht="14.25">
+      <c r="A40" s="32"/>
+      <c r="B40" s="33"/>
+      <c r="C40" s="33"/>
+      <c r="D40" s="34"/>
+      <c r="E40" s="33"/>
+      <c r="F40" s="33"/>
+      <c r="G40" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -1786,7 +1821,7 @@
     <mergeCell ref="E3:G3"/>
     <mergeCell ref="A19:G19"/>
     <mergeCell ref="A26:G26"/>
-    <mergeCell ref="A35:G35"/>
+    <mergeCell ref="A36:G36"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
trips: offer redirect, Step-10.2/15.2 pickup Notes, drop redundant Paid line
- offer_create now redirects the carrier to their new offer's detail page
  (?offer=<id>#offer-detail) instead of jumping to #travel-plans.
- Copy Step-10.2 (all roles) and Step-15.2 (buyer date) pickup Notes from the
  sheet; split the carrier/proxy ready_for_pickup pickup_selected branches.
- Remove the redundant "Paid — Your balance is settled" line from the buyer's
  ready_for_pickup Notes (kept the overpaid-refund notice).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proxybuying-obsidian/AI-Context/references/UserAndSystemStepsRelationship.xlsx
+++ b/proxybuying-obsidian/AI-Context/references/UserAndSystemStepsRelationship.xlsx
@@ -355,7 +355,7 @@
     <t>15.2</t>
   </si>
   <si>
-    <t xml:space="preserve">You have reviewed and received the package. Transaction closed</t>
+    <t xml:space="preserve">You have reviewed and received the package on &lt;date, time&gt;. Transaction closed</t>
   </si>
   <si>
     <t xml:space="preserve">Package collected by the Buyer. Your payout will be disbursed within 24 hours.</t>
@@ -1780,11 +1780,11 @@
         <v>110</v>
       </c>
     </row>
-    <row r="39" ht="42.75">
-      <c r="A39" s="26" t="s">
+    <row r="39" ht="57">
+      <c r="A39" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="B39" s="26" t="s">
+      <c r="B39" s="9" t="s">
         <v>111</v>
       </c>
       <c r="C39" s="9" t="s">
@@ -1793,7 +1793,7 @@
       <c r="D39" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="E39" s="12" t="s">
+      <c r="E39" s="22" t="s">
         <v>112</v>
       </c>
       <c r="F39" s="12" t="s">

</xml_diff>

<commit_message>
docs: update UserAndSystemStepsRelationship reference (Step-1.1/2-3 buyer-CRUD)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proxybuying-obsidian/AI-Context/references/UserAndSystemStepsRelationship.xlsx
+++ b/proxybuying-obsidian/AI-Context/references/UserAndSystemStepsRelationship.xlsx
@@ -6,7 +6,7 @@
     <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
   </sheets>
   <calcPr/>
   <extLst>
@@ -15,6 +15,37 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={CFFA49ED-4450-354E-22CF-5ACF75A6C676}</author>
+  </authors>
+  <commentList>
+    <comment ref="E8" authorId="0" xr:uid="{CFFA49ED-4450-354E-22CF-5ACF75A6C676}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+          </rPr>
+          <t>opa:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">
+Update wordings
+</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="114">
   <si>
@@ -78,7 +109,7 @@
     <t xml:space="preserve">Clicked on "Process Estimate" button on "Action" column on "My Proxy Buying" table</t>
   </si>
   <si>
-    <t xml:space="preserve">Please fill in all required data. After you click "Send Estimate" Buyer will be notified.</t>
+    <t xml:space="preserve">Please fill in all required data. After you click "Send Estimate" Buyer will be notified. Use the Chat Box to discuss with Buyer on ordered products issues (out-of-stock, shortage quantity, etc.)</t>
   </si>
   <si>
     <t>2.2</t>
@@ -87,7 +118,7 @@
     <t xml:space="preserve">Clicked on "Send Estimate"</t>
   </si>
   <si>
-    <t xml:space="preserve">Proxy Buyer has sent the estimate. Please Accept or Reject it. Use the Chat Box if you want to negotiate the Margin with Proxy Buyer.</t>
+    <t xml:space="preserve">Proxy Buyer has sent the estimate. Please Accept, Edit, or Reject it. Editing your order sends it back to the Proxy Buyer to re-estimate. Use the Chat Box if you want to negotiate the Margin with Proxy Buyer.</t>
   </si>
   <si>
     <t xml:space="preserve">Estimate Sent, waiting for Buyer to Accept it. Use the Chat Box to check if Buyer is asking to negotiate the Margin. You still be able to edit the Margin before Buyer Accepting or Rejecting your estimate.</t>
@@ -451,7 +482,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="30">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -493,11 +524,8 @@
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -505,16 +533,7 @@
     <xf fontId="0" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf fontId="0" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
@@ -535,9 +554,6 @@
     </xf>
     <xf fontId="1" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="164" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -564,6 +580,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="opa" id="{8DC25E0B-C16D-9521-27F4-677E169D6E97}" userId="opa" providerId="Teamlab"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1044,6 +1066,15 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="E8" dT="2026-07-06T03:30:59.03Z" personId="{8DC25E0B-C16D-9521-27F4-677E169D6E97}" id="{CFFA49ED-4450-354E-22CF-5ACF75A6C676}" done="1">
+    <text xml:space="preserve">Update wordings
+</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -1155,7 +1186,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" ht="71.25">
+    <row r="7" ht="99.75">
       <c r="A7" s="9">
         <v>2</v>
       </c>
@@ -1191,10 +1222,10 @@
       <c r="D8" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="11" t="s">
         <v>24</v>
       </c>
       <c r="G8" s="12" t="s">
@@ -1214,10 +1245,10 @@
       <c r="D9" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="E9" s="15" t="s">
+      <c r="E9" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="13" t="s">
         <v>27</v>
       </c>
       <c r="G9" s="12" t="s">
@@ -1234,25 +1265,25 @@
       <c r="C10" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D10" s="16" t="s">
+      <c r="D10" s="10" t="s">
         <v>29</v>
       </c>
       <c r="E10" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="13" t="s">
         <v>27</v>
       </c>
       <c r="G10" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="L10" s="17" t="s">
+      <c r="L10" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="M10" s="17" t="s">
+      <c r="M10" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="N10" s="17" t="s">
+      <c r="N10" s="16" t="s">
         <v>30</v>
       </c>
     </row>
@@ -1292,7 +1323,7 @@
       <c r="D12" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="E12" s="14" t="s">
+      <c r="E12" s="11" t="s">
         <v>39</v>
       </c>
       <c r="F12" s="11" t="s">
@@ -1306,7 +1337,7 @@
       <c r="A13" s="9">
         <v>5</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="17" t="s">
         <v>42</v>
       </c>
       <c r="C13" s="9" t="s">
@@ -1315,13 +1346,13 @@
       <c r="D13" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="E13" s="19" t="s">
+      <c r="E13" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="F13" s="19" t="s">
+      <c r="F13" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="G13" s="19" t="s">
+      <c r="G13" s="15" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1329,7 +1360,7 @@
       <c r="A14" s="9">
         <v>5</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="17" t="s">
         <v>46</v>
       </c>
       <c r="C14" s="9" t="s">
@@ -1338,13 +1369,13 @@
       <c r="D14" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="E14" s="20" t="s">
+      <c r="E14" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="F14" s="14" t="s">
+      <c r="F14" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="G14" s="15" t="s">
+      <c r="G14" s="13" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1352,7 +1383,7 @@
       <c r="A15" s="9">
         <v>6</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="17" t="s">
         <v>52</v>
       </c>
       <c r="C15" s="10" t="s">
@@ -1361,7 +1392,7 @@
       <c r="D15" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="E15" s="21" t="s">
+      <c r="E15" s="18" t="s">
         <v>49</v>
       </c>
       <c r="F15" s="11" t="s">
@@ -1375,7 +1406,7 @@
       <c r="A16" s="9">
         <v>6</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="B16" s="17" t="s">
         <v>55</v>
       </c>
       <c r="C16" s="10" t="s">
@@ -1384,13 +1415,13 @@
       <c r="D16" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="E16" s="22" t="s">
+      <c r="E16" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="F16" s="14" t="s">
+      <c r="F16" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="G16" s="14" t="s">
+      <c r="G16" s="11" t="s">
         <v>59</v>
       </c>
     </row>
@@ -1398,7 +1429,7 @@
       <c r="A17" s="9">
         <v>7</v>
       </c>
-      <c r="B17" s="18">
+      <c r="B17" s="17">
         <v>7</v>
       </c>
       <c r="C17" s="9" t="s">
@@ -1407,10 +1438,10 @@
       <c r="D17" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="E17" s="21" t="s">
+      <c r="E17" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="F17" s="21" t="s">
+      <c r="F17" s="18" t="s">
         <v>62</v>
       </c>
       <c r="G17" s="13" t="s">
@@ -1438,19 +1469,19 @@
       <c r="G19" s="6"/>
     </row>
     <row r="20" ht="14.25">
-      <c r="A20" s="23"/>
-      <c r="B20" s="23"/>
-      <c r="C20" s="23"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="23"/>
-      <c r="G20" s="23"/>
+      <c r="A20" s="19"/>
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="19"/>
     </row>
     <row r="21" ht="99.75">
       <c r="A21" s="9">
         <v>8</v>
       </c>
-      <c r="B21" s="18" t="s">
+      <c r="B21" s="17" t="s">
         <v>65</v>
       </c>
       <c r="C21" s="9" t="s">
@@ -1459,13 +1490,13 @@
       <c r="D21" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="E21" s="21" t="s">
+      <c r="E21" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="F21" s="21" t="s">
+      <c r="F21" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="G21" s="19" t="s">
+      <c r="G21" s="15" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1473,7 +1504,7 @@
       <c r="A22" s="9">
         <v>8</v>
       </c>
-      <c r="B22" s="18" t="s">
+      <c r="B22" s="17" t="s">
         <v>68</v>
       </c>
       <c r="C22" s="9" t="s">
@@ -1482,13 +1513,13 @@
       <c r="D22" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="E22" s="22" t="s">
+      <c r="E22" s="12" t="s">
         <v>70</v>
       </c>
       <c r="F22" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="G22" s="24" t="s">
+      <c r="G22" s="20" t="s">
         <v>72</v>
       </c>
     </row>
@@ -1496,7 +1527,7 @@
       <c r="A23" s="9">
         <v>9</v>
       </c>
-      <c r="B23" s="18" t="s">
+      <c r="B23" s="17" t="s">
         <v>73</v>
       </c>
       <c r="C23" s="9" t="s">
@@ -1519,7 +1550,7 @@
       <c r="A24" s="9">
         <v>9</v>
       </c>
-      <c r="B24" s="18" t="s">
+      <c r="B24" s="17" t="s">
         <v>77</v>
       </c>
       <c r="C24" s="9" t="s">
@@ -1528,24 +1559,24 @@
       <c r="D24" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="E24" s="25" t="s">
+      <c r="E24" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="F24" s="25" t="s">
+      <c r="F24" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="G24" s="25" t="s">
+      <c r="G24" s="21" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="25" ht="14.25">
-      <c r="A25" s="26"/>
-      <c r="B25" s="23"/>
-      <c r="C25" s="23"/>
-      <c r="D25" s="27"/>
-      <c r="E25" s="23"/>
-      <c r="F25" s="23"/>
-      <c r="G25" s="23"/>
+      <c r="A25" s="22"/>
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="23"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="19"/>
+      <c r="G25" s="19"/>
     </row>
     <row r="26" ht="14.25">
       <c r="A26" s="6" t="s">
@@ -1559,19 +1590,19 @@
       <c r="G26" s="6"/>
     </row>
     <row r="27" ht="14.25">
-      <c r="A27" s="26"/>
-      <c r="B27" s="23"/>
-      <c r="C27" s="23"/>
-      <c r="D27" s="27"/>
-      <c r="E27" s="23"/>
-      <c r="F27" s="23"/>
-      <c r="G27" s="23"/>
+      <c r="A27" s="22"/>
+      <c r="B27" s="19"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="23"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="19"/>
+      <c r="G27" s="19"/>
     </row>
     <row r="28" ht="57">
-      <c r="A28" s="28" t="s">
+      <c r="A28" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="B28" s="18" t="s">
+      <c r="B28" s="17" t="s">
         <v>82</v>
       </c>
       <c r="C28" s="9" t="s">
@@ -1580,13 +1611,13 @@
       <c r="D28" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="E28" s="29" t="s">
+      <c r="E28" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="F28" s="29" t="s">
+      <c r="F28" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="G28" s="29" t="s">
+      <c r="G28" s="25" t="s">
         <v>86</v>
       </c>
     </row>
@@ -1594,13 +1625,13 @@
       <c r="A29" s="9">
         <v>11</v>
       </c>
-      <c r="B29" s="18">
+      <c r="B29" s="17">
         <v>11</v>
       </c>
       <c r="C29" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="D29" s="16" t="s">
+      <c r="D29" s="10" t="s">
         <v>87</v>
       </c>
       <c r="E29" s="12" t="s">
@@ -1617,7 +1648,7 @@
       <c r="A30" s="9">
         <v>12</v>
       </c>
-      <c r="B30" s="18">
+      <c r="B30" s="17">
         <v>12</v>
       </c>
       <c r="C30" s="9" t="s">
@@ -1640,13 +1671,13 @@
       <c r="A31" s="9">
         <v>13</v>
       </c>
-      <c r="B31" s="18">
+      <c r="B31" s="17">
         <v>13</v>
       </c>
       <c r="C31" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="D31" s="16" t="s">
+      <c r="D31" s="10" t="s">
         <v>93</v>
       </c>
       <c r="E31" s="12" t="s">
@@ -1663,7 +1694,7 @@
       <c r="A32" s="9">
         <v>14</v>
       </c>
-      <c r="B32" s="18">
+      <c r="B32" s="17">
         <v>14</v>
       </c>
       <c r="C32" s="9" t="s">
@@ -1686,7 +1717,7 @@
       <c r="A33" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="B33" s="18" t="s">
+      <c r="B33" s="17" t="s">
         <v>100</v>
       </c>
       <c r="C33" s="9" t="s">
@@ -1695,13 +1726,13 @@
       <c r="D33" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="E33" s="22" t="s">
+      <c r="E33" s="12" t="s">
         <v>101</v>
       </c>
       <c r="F33" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="G33" s="22" t="s">
+      <c r="G33" s="12" t="s">
         <v>102</v>
       </c>
     </row>
@@ -1709,22 +1740,22 @@
       <c r="A34" s="9">
         <v>16</v>
       </c>
-      <c r="B34" s="18">
+      <c r="B34" s="17">
         <v>16</v>
       </c>
-      <c r="C34" s="30" t="s">
+      <c r="C34" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="D34" s="16" t="s">
+      <c r="D34" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="E34" s="22" t="s">
+      <c r="E34" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="F34" s="22" t="s">
+      <c r="F34" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="G34" s="22" t="s">
+      <c r="G34" s="12" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1733,9 +1764,9 @@
       <c r="B35" s="9"/>
       <c r="C35" s="9"/>
       <c r="D35" s="10"/>
-      <c r="E35" s="23"/>
-      <c r="F35" s="23"/>
-      <c r="G35" s="23"/>
+      <c r="E35" s="19"/>
+      <c r="F35" s="19"/>
+      <c r="G35" s="19"/>
     </row>
     <row r="36" ht="14.25">
       <c r="A36" s="6" t="s">
@@ -1749,19 +1780,19 @@
       <c r="G36" s="6"/>
     </row>
     <row r="37" ht="14.25">
-      <c r="A37" s="26"/>
-      <c r="B37" s="23"/>
-      <c r="C37" s="23"/>
-      <c r="D37" s="27"/>
-      <c r="E37" s="23"/>
-      <c r="F37" s="23"/>
-      <c r="G37" s="23"/>
+      <c r="A37" s="22"/>
+      <c r="B37" s="19"/>
+      <c r="C37" s="19"/>
+      <c r="D37" s="23"/>
+      <c r="E37" s="19"/>
+      <c r="F37" s="19"/>
+      <c r="G37" s="19"/>
     </row>
     <row r="38" ht="57">
-      <c r="A38" s="31" t="s">
+      <c r="A38" s="26" t="s">
         <v>107</v>
       </c>
-      <c r="B38" s="31" t="s">
+      <c r="B38" s="26" t="s">
         <v>107</v>
       </c>
       <c r="C38" s="9" t="s">
@@ -1793,7 +1824,7 @@
       <c r="D39" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="E39" s="22" t="s">
+      <c r="E39" s="12" t="s">
         <v>112</v>
       </c>
       <c r="F39" s="12" t="s">
@@ -1804,13 +1835,13 @@
       </c>
     </row>
     <row r="40" ht="14.25">
-      <c r="A40" s="32"/>
-      <c r="B40" s="33"/>
-      <c r="C40" s="33"/>
-      <c r="D40" s="34"/>
-      <c r="E40" s="33"/>
-      <c r="F40" s="33"/>
-      <c r="G40" s="33"/>
+      <c r="A40" s="27"/>
+      <c r="B40" s="28"/>
+      <c r="C40" s="28"/>
+      <c r="D40" s="29"/>
+      <c r="E40" s="28"/>
+      <c r="F40" s="28"/>
+      <c r="G40" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -1827,5 +1858,6 @@
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="0" copies="1"/>
   <headerFooter/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>